<commit_message>
- I don't exactly remember - Test stuff for bandit camps being always visible and attempt at neutral arena spectators spawned by prop
</commit_message>
<xml_diff>
--- a/Items+Troops Spreadsheets/HYW Item Balance.xlsx
+++ b/Items+Troops Spreadsheets/HYW Item Balance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yoann\OneDrive\Ambiente de Trabalho\Deeds_Modsys\Items+Troops Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A4172D8-B951-4981-94D3-8902C9758949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C70D800A-78CC-4A8A-B472-BD5EA0CA30B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" firstSheet="9" activeTab="15" xr2:uid="{B36B220B-AFFD-40C9-B18F-2948A113413C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="8" activeTab="15" xr2:uid="{B36B220B-AFFD-40C9-B18F-2948A113413C}"/>
   </bookViews>
   <sheets>
     <sheet name="Maces" sheetId="1" r:id="rId1"/>
@@ -19,16 +19,16 @@
     <sheet name="Bastard &amp; Twohanded Swords" sheetId="4" r:id="rId4"/>
     <sheet name="Pikes &amp; Halberds" sheetId="5" r:id="rId5"/>
     <sheet name="Halberds" sheetId="14" r:id="rId6"/>
-    <sheet name="Feuil1" sheetId="15" r:id="rId7"/>
-    <sheet name="Forks &amp; Fauchards" sheetId="8" r:id="rId8"/>
-    <sheet name="Glaives &amp; Couteau" sheetId="13" r:id="rId9"/>
-    <sheet name="Spears &amp; Lances" sheetId="9" r:id="rId10"/>
-    <sheet name="Pollaxes" sheetId="12" r:id="rId11"/>
-    <sheet name="Bows &amp; Crossbows" sheetId="6" r:id="rId12"/>
-    <sheet name="Horses" sheetId="7" r:id="rId13"/>
-    <sheet name="Arrows &amp; Bolts" sheetId="10" r:id="rId14"/>
-    <sheet name="Shields" sheetId="11" r:id="rId15"/>
-    <sheet name="Helmets" sheetId="16" r:id="rId16"/>
+    <sheet name="Forks &amp; Fauchards" sheetId="8" r:id="rId7"/>
+    <sheet name="Glaives &amp; Couteau" sheetId="13" r:id="rId8"/>
+    <sheet name="Spears &amp; Lances" sheetId="9" r:id="rId9"/>
+    <sheet name="Pollaxes" sheetId="12" r:id="rId10"/>
+    <sheet name="Bows &amp; Crossbows" sheetId="6" r:id="rId11"/>
+    <sheet name="Horses" sheetId="7" r:id="rId12"/>
+    <sheet name="Arrows &amp; Bolts" sheetId="10" r:id="rId13"/>
+    <sheet name="Shields" sheetId="11" r:id="rId14"/>
+    <sheet name="Helmets" sheetId="16" r:id="rId15"/>
+    <sheet name="Armour" sheetId="15" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="465">
   <si>
     <t>ID</t>
   </si>
@@ -1383,6 +1383,66 @@
   </si>
   <si>
     <t>h_great_sallet_visor</t>
+  </si>
+  <si>
+    <t>Leg Armour</t>
+  </si>
+  <si>
+    <t>a_english_plate_1445_1450_gilded</t>
+  </si>
+  <si>
+    <t>a_english_plate_1445_1450</t>
+  </si>
+  <si>
+    <t>a_english_plate_1435_1450_gilded</t>
+  </si>
+  <si>
+    <t>a_english_plate_1435_1450</t>
+  </si>
+  <si>
+    <t>a_english_plate_1430_1445_gilded</t>
+  </si>
+  <si>
+    <t>a_english_plate_1430_1445</t>
+  </si>
+  <si>
+    <t>a_english_plate_1415_a_gilded_besagews</t>
+  </si>
+  <si>
+    <t>a_english_plate_1415_a_gilded</t>
+  </si>
+  <si>
+    <t>a_english_plate_1415_a_besagews</t>
+  </si>
+  <si>
+    <t>a_english_plate_1415_a</t>
+  </si>
+  <si>
+    <t>a_plate_kastenbrust_a</t>
+  </si>
+  <si>
+    <t>a_continental_plate_a</t>
+  </si>
+  <si>
+    <t>a_padded_over_plate_sleeved_deco_1</t>
+  </si>
+  <si>
+    <t>a_padded_over_plate_sleeved_1_custom</t>
+  </si>
+  <si>
+    <t>a_padded_over_plate_shortsleeved_1_custom</t>
+  </si>
+  <si>
+    <t>a_padded_over_plate_sleeveless_1_custom</t>
+  </si>
+  <si>
+    <t>a_plate_german_covered_fauld_custom</t>
+  </si>
+  <si>
+    <t>a_english_plate_1415_heraldic</t>
+  </si>
+  <si>
+    <t>a_jupon_heraldic</t>
   </si>
 </sst>
 </file>
@@ -1404,7 +1464,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1519,6 +1579,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -1590,7 +1668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1643,11 +1721,46 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="29">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1874,18 +1987,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F5046EE-3462-4861-8BA7-BDFE936F9817}" name="Tableau1" displayName="Tableau1" ref="A1:I9" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F5046EE-3462-4861-8BA7-BDFE936F9817}" name="Tableau1" displayName="Tableau1" ref="A1:I9" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26">
   <autoFilter ref="A1:I9" xr:uid="{C03180B4-6AED-435F-B389-4A4563BC2CC7}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C9803FB6-EDE5-4D36-AE31-771E624ABD45}" name="Native" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{5FC1EA44-BFAD-4BBC-B86E-2A3CF8B5EE66}" name="Price" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{01474069-2C07-4B0D-BCD4-BCBEA8815443}" name="Weight" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{90286B08-5EC7-4290-B829-6A962FFA020D}" name="Hitpoints" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{BEB87F5A-2E44-49CC-B818-CB41CAE1540E}" name="Armor" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{1FC9649F-49E2-4557-9365-90302BBA23F5}" name="Speed" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{9DBEE228-7BC6-4A16-9AEA-276D82F520AF}" name="Width " dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{F49F7FEF-63B8-416A-B721-00BC45756836}" name="Height" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{2B135CC7-F1ED-468C-AA68-F96B873B45CB}" name="Colonne1" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{C9803FB6-EDE5-4D36-AE31-771E624ABD45}" name="Native" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{5FC1EA44-BFAD-4BBC-B86E-2A3CF8B5EE66}" name="Price" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{01474069-2C07-4B0D-BCD4-BCBEA8815443}" name="Weight" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{90286B08-5EC7-4290-B829-6A962FFA020D}" name="Hitpoints" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{BEB87F5A-2E44-49CC-B818-CB41CAE1540E}" name="Armor" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{1FC9649F-49E2-4557-9365-90302BBA23F5}" name="Speed" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{9DBEE228-7BC6-4A16-9AEA-276D82F520AF}" name="Width " dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{F49F7FEF-63B8-416A-B721-00BC45756836}" name="Height" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{2B135CC7-F1ED-468C-AA68-F96B873B45CB}" name="Colonne1" dataDxfId="17">
       <calculatedColumnFormula>((Tableau1[[#This Row],[Hitpoints]]*Tableau1[[#This Row],[Armor]]*2)+(Tableau1[[#This Row],[Width ]]*Tableau1[[#This Row],[Height]]*2)-(Tableau1[[#This Row],[Speed]]*Tableau1[[#This Row],[Weight]]))/100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1894,16 +2007,30 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D59FB3B4-EC06-4D73-9946-6BFE2C2CCBE1}" name="Tableau2" displayName="Tableau2" ref="A7:E71" headerRowDxfId="12" dataDxfId="11" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D59FB3B4-EC06-4D73-9946-6BFE2C2CCBE1}" name="Tableau2" displayName="Tableau2" ref="A7:E71" headerRowDxfId="16" dataDxfId="15" tableBorderDxfId="14">
   <autoFilter ref="A7:E71" xr:uid="{D59FB3B4-EC06-4D73-9946-6BFE2C2CCBE1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{21613AAF-B76C-4060-ACB4-4C1DBB9C3B0B}" name="ID" totalsRowLabel="Total" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{21CBE435-491F-46CE-AC9C-F4DC60BC75DA}" name="Price" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{0C92D438-FF0E-4E4D-A49D-F1E5D03F952C}" name="Weight" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{974C9707-BBDC-49A3-A159-86CDDB7C55BC}" name="Head Armour" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{53D86C19-4C70-4593-BC24-2F9BB8ACF6DE}" name="Body Armour" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{21613AAF-B76C-4060-ACB4-4C1DBB9C3B0B}" name="ID" totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{21CBE435-491F-46CE-AC9C-F4DC60BC75DA}" name="Price" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{0C92D438-FF0E-4E4D-A49D-F1E5D03F952C}" name="Weight" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{974C9707-BBDC-49A3-A159-86CDDB7C55BC}" name="Head Armour" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{53D86C19-4C70-4593-BC24-2F9BB8ACF6DE}" name="Body Armour" totalsRowFunction="sum" dataDxfId="5" totalsRowDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C9EC37F5-71DB-414B-B7B1-A485339ED55A}" name="Tableau3" displayName="Tableau3" ref="A1:E23" totalsRowShown="0">
+  <autoFilter ref="A1:E23" xr:uid="{C9EC37F5-71DB-414B-B7B1-A485339ED55A}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{C62F6CC2-BCA5-4784-B561-AFB847D1F169}" name="ID" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{201E955D-2542-4BE2-A720-83AF4EB55A51}" name="Price" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{AAE4B832-72D5-4564-AD22-F2C578CF0651}" name="Weight" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{ED953D68-A757-4D7D-9D80-C0AE6B3FDCB5}" name="Body Armour"/>
+    <tableColumn id="5" xr3:uid="{6C3E02DF-366F-42A5-8D7A-AA5CA34962BD}" name="Leg Armour" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2786,773 +2913,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{270FCD42-7C0A-42FB-9872-27F0BB063FAE}">
-  <dimension ref="A1:I32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="26.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="6">
-        <v>134</v>
-      </c>
-      <c r="D2" s="4">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E2" s="7">
-        <v>0</v>
-      </c>
-      <c r="F2" s="5">
-        <v>99</v>
-      </c>
-      <c r="G2" s="3">
-        <v>107</v>
-      </c>
-      <c r="H2" s="1">
-        <v>37</v>
-      </c>
-      <c r="I2">
-        <f>SUM(D2:H2)*0.55</f>
-        <v>134.255</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="6">
-        <v>144</v>
-      </c>
-      <c r="D3" s="4">
-        <v>1.3</v>
-      </c>
-      <c r="E3" s="7">
-        <v>0</v>
-      </c>
-      <c r="F3" s="5">
-        <v>97</v>
-      </c>
-      <c r="G3" s="3">
-        <v>128</v>
-      </c>
-      <c r="H3" s="1">
-        <v>36</v>
-      </c>
-      <c r="I3">
-        <f>SUM(D3:H3)*0.55</f>
-        <v>144.26500000000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="6">
-        <v>146</v>
-      </c>
-      <c r="D4" s="4">
-        <v>1.3</v>
-      </c>
-      <c r="E4" s="7">
-        <v>0</v>
-      </c>
-      <c r="F4" s="5">
-        <v>97</v>
-      </c>
-      <c r="G4" s="3">
-        <v>132</v>
-      </c>
-      <c r="H4" s="1">
-        <v>36</v>
-      </c>
-      <c r="I4">
-        <f>SUM(D4:H4)*0.55</f>
-        <v>146.46500000000003</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="6">
-        <v>165</v>
-      </c>
-      <c r="D5" s="4">
-        <v>1.4</v>
-      </c>
-      <c r="E5" s="7">
-        <v>0</v>
-      </c>
-      <c r="F5" s="5">
-        <v>96</v>
-      </c>
-      <c r="G5" s="3">
-        <v>142</v>
-      </c>
-      <c r="H5" s="1">
-        <v>35</v>
-      </c>
-      <c r="I5">
-        <f>SUM(D5:H5)*0.6</f>
-        <v>164.64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="6">
-        <v>166</v>
-      </c>
-      <c r="D6" s="4">
-        <v>1.4</v>
-      </c>
-      <c r="E6" s="7">
-        <v>0</v>
-      </c>
-      <c r="F6" s="5">
-        <v>96</v>
-      </c>
-      <c r="G6" s="3">
-        <v>144</v>
-      </c>
-      <c r="H6" s="1">
-        <v>35</v>
-      </c>
-      <c r="I6">
-        <f>SUM(D6:H6)*0.6</f>
-        <v>165.83999999999997</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="6">
-        <v>168</v>
-      </c>
-      <c r="D7" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="E7" s="7">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>95</v>
-      </c>
-      <c r="G7" s="3">
-        <v>149</v>
-      </c>
-      <c r="H7" s="1">
-        <v>34</v>
-      </c>
-      <c r="I7">
-        <f>SUM(D7:H7)*0.6</f>
-        <v>167.7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="6">
-        <v>229</v>
-      </c>
-      <c r="D8" s="4">
-        <v>2</v>
-      </c>
-      <c r="E8" s="7">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5">
-        <v>90</v>
-      </c>
-      <c r="G8" s="3">
-        <v>204</v>
-      </c>
-      <c r="H8" s="1">
-        <v>31</v>
-      </c>
-      <c r="I8">
-        <f>SUM(D8:H8)*0.7</f>
-        <v>228.89999999999998</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="6">
-        <v>117</v>
-      </c>
-      <c r="D9" s="4">
-        <v>1</v>
-      </c>
-      <c r="E9" s="7">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>100</v>
-      </c>
-      <c r="G9" s="3">
-        <v>95</v>
-      </c>
-      <c r="H9" s="1">
-        <v>38</v>
-      </c>
-      <c r="I9">
-        <f>SUM(D9:H9)*0.5</f>
-        <v>117</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="6">
-        <v>87</v>
-      </c>
-      <c r="D11" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="E11" s="7">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>87</v>
-      </c>
-      <c r="G11" s="3">
-        <v>135</v>
-      </c>
-      <c r="H11" s="1">
-        <v>26</v>
-      </c>
-      <c r="I11">
-        <f>SUM(D11:H11)*0.35</f>
-        <v>87.324999999999989</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="6">
-        <v>84</v>
-      </c>
-      <c r="D12" s="4">
-        <v>1.4</v>
-      </c>
-      <c r="E12" s="7">
-        <v>0</v>
-      </c>
-      <c r="F12" s="5">
-        <v>88</v>
-      </c>
-      <c r="G12" s="3">
-        <v>126</v>
-      </c>
-      <c r="H12" s="1">
-        <v>25</v>
-      </c>
-      <c r="I12">
-        <f>SUM(D12:H12)*0.35</f>
-        <v>84.14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="6">
-        <v>142</v>
-      </c>
-      <c r="D13" s="4">
-        <v>2</v>
-      </c>
-      <c r="E13" s="7">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5">
-        <v>84</v>
-      </c>
-      <c r="G13" s="3">
-        <v>168</v>
-      </c>
-      <c r="H13" s="1">
-        <v>31</v>
-      </c>
-      <c r="I13">
-        <f>SUM(D13:H13)*0.5</f>
-        <v>142.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="6">
-        <v>285</v>
-      </c>
-      <c r="D15" s="4">
-        <v>3</v>
-      </c>
-      <c r="E15" s="7">
-        <v>9</v>
-      </c>
-      <c r="F15" s="5">
-        <v>84</v>
-      </c>
-      <c r="G15" s="3">
-        <v>355</v>
-      </c>
-      <c r="H15" s="1">
-        <v>25</v>
-      </c>
-      <c r="I15">
-        <f>SUM(D15:H15)*0.6</f>
-        <v>285.59999999999997</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="6">
-        <v>214</v>
-      </c>
-      <c r="D16" s="4">
-        <v>2.5</v>
-      </c>
-      <c r="E16" s="7">
-        <v>9</v>
-      </c>
-      <c r="F16" s="5">
-        <v>92</v>
-      </c>
-      <c r="G16" s="3">
-        <v>175</v>
-      </c>
-      <c r="H16" s="1">
-        <v>27</v>
-      </c>
-      <c r="I16">
-        <f>SUM(D16:H16)*0.7</f>
-        <v>213.85</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="6">
-        <v>224</v>
-      </c>
-      <c r="D17" s="4">
-        <v>2.4</v>
-      </c>
-      <c r="E17" s="7">
-        <v>9</v>
-      </c>
-      <c r="F17" s="5">
-        <v>90</v>
-      </c>
-      <c r="G17" s="3">
-        <v>190</v>
-      </c>
-      <c r="H17" s="1">
-        <v>29</v>
-      </c>
-      <c r="I17">
-        <f>SUM(D17:H17)*0.7</f>
-        <v>224.27999999999997</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="6">
-        <v>320</v>
-      </c>
-      <c r="D19" s="4">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="E19" s="7">
-        <v>12</v>
-      </c>
-      <c r="F19" s="5">
-        <v>82</v>
-      </c>
-      <c r="G19" s="3">
-        <v>267</v>
-      </c>
-      <c r="H19" s="1">
-        <v>35</v>
-      </c>
-      <c r="I19">
-        <f t="shared" ref="I19:I24" si="0">SUM(D19:H19)*0.8</f>
-        <v>320.32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="6">
-        <v>286</v>
-      </c>
-      <c r="D20" s="4">
-        <v>4</v>
-      </c>
-      <c r="E20" s="7">
-        <v>12</v>
-      </c>
-      <c r="F20" s="5">
-        <v>85</v>
-      </c>
-      <c r="G20" s="3">
-        <v>226</v>
-      </c>
-      <c r="H20" s="1">
-        <v>31</v>
-      </c>
-      <c r="I20">
-        <f t="shared" si="0"/>
-        <v>286.40000000000003</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="6">
-        <v>307</v>
-      </c>
-      <c r="D21" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E21" s="7">
-        <v>12</v>
-      </c>
-      <c r="F21" s="5">
-        <v>83</v>
-      </c>
-      <c r="G21" s="3">
-        <v>253</v>
-      </c>
-      <c r="H21" s="1">
-        <v>32</v>
-      </c>
-      <c r="I21">
-        <f t="shared" si="0"/>
-        <v>307.36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="6">
-        <v>307</v>
-      </c>
-      <c r="D22" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E22" s="7">
-        <v>12</v>
-      </c>
-      <c r="F22" s="5">
-        <v>83</v>
-      </c>
-      <c r="G22" s="3">
-        <v>253</v>
-      </c>
-      <c r="H22" s="1">
-        <v>32</v>
-      </c>
-      <c r="I22">
-        <f t="shared" si="0"/>
-        <v>307.36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="6">
-        <v>308</v>
-      </c>
-      <c r="D23" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E23" s="7">
-        <v>12</v>
-      </c>
-      <c r="F23" s="5">
-        <v>83</v>
-      </c>
-      <c r="G23" s="3">
-        <v>252</v>
-      </c>
-      <c r="H23" s="1">
-        <v>34</v>
-      </c>
-      <c r="I23">
-        <f t="shared" si="0"/>
-        <v>308.16000000000003</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="6">
-        <v>296</v>
-      </c>
-      <c r="D24" s="4">
-        <v>4.3</v>
-      </c>
-      <c r="E24" s="7">
-        <v>12</v>
-      </c>
-      <c r="F24" s="5">
-        <v>83</v>
-      </c>
-      <c r="G24" s="3">
-        <v>241</v>
-      </c>
-      <c r="H24" s="1">
-        <v>30</v>
-      </c>
-      <c r="I24">
-        <f t="shared" si="0"/>
-        <v>296.24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="6">
-        <v>308</v>
-      </c>
-      <c r="D26" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E26" s="7">
-        <v>12</v>
-      </c>
-      <c r="F26" s="5">
-        <v>83</v>
-      </c>
-      <c r="G26" s="3">
-        <v>252</v>
-      </c>
-      <c r="H26" s="1">
-        <v>34</v>
-      </c>
-      <c r="I26">
-        <f>SUM(D26:H26)*0.8</f>
-        <v>308.16000000000003</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="6">
-        <v>308</v>
-      </c>
-      <c r="D27" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E27" s="7">
-        <v>12</v>
-      </c>
-      <c r="F27" s="5">
-        <v>83</v>
-      </c>
-      <c r="G27" s="3">
-        <v>252</v>
-      </c>
-      <c r="H27" s="1">
-        <v>34</v>
-      </c>
-      <c r="I27">
-        <f>SUM(D27:H27)*0.8</f>
-        <v>308.16000000000003</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="6">
-        <v>320</v>
-      </c>
-      <c r="D28" s="4">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="E28" s="7">
-        <v>12</v>
-      </c>
-      <c r="F28" s="5">
-        <v>82</v>
-      </c>
-      <c r="G28" s="3">
-        <v>267</v>
-      </c>
-      <c r="H28" s="1">
-        <v>35</v>
-      </c>
-      <c r="I28">
-        <f>SUM(D28:H28)*0.8</f>
-        <v>320.32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="6">
-        <v>308</v>
-      </c>
-      <c r="D30" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E30" s="7">
-        <v>12</v>
-      </c>
-      <c r="F30" s="5">
-        <v>83</v>
-      </c>
-      <c r="G30" s="3">
-        <v>252</v>
-      </c>
-      <c r="H30" s="1">
-        <v>34</v>
-      </c>
-      <c r="I30">
-        <f>SUM(D30:H30)*0.8</f>
-        <v>308.16000000000003</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="6">
-        <v>308</v>
-      </c>
-      <c r="D31" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E31" s="7">
-        <v>12</v>
-      </c>
-      <c r="F31" s="5">
-        <v>83</v>
-      </c>
-      <c r="G31" s="3">
-        <v>252</v>
-      </c>
-      <c r="H31" s="1">
-        <v>34</v>
-      </c>
-      <c r="I31">
-        <f>SUM(D31:H31)*0.8</f>
-        <v>308.16000000000003</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="6">
-        <v>308</v>
-      </c>
-      <c r="D32" s="4">
-        <v>4.2</v>
-      </c>
-      <c r="E32" s="7">
-        <v>12</v>
-      </c>
-      <c r="F32" s="5">
-        <v>83</v>
-      </c>
-      <c r="G32" s="3">
-        <v>252</v>
-      </c>
-      <c r="H32" s="1">
-        <v>34</v>
-      </c>
-      <c r="I32">
-        <f>SUM(D32:H32)*0.8</f>
-        <v>308.16000000000003</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C18765D9-5E60-43F7-8EAE-7692D37C4247}">
   <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4232,7 +3592,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96551E4B-D0DF-400F-B6DB-43F70FA502C4}">
   <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4897,7 +4257,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00DAD396-9A3B-4E45-8468-1404C7D6E830}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5189,7 +4549,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3C8FEF-B598-4AEC-9E3E-97CE35ABD837}">
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5442,7 +4802,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6EE9141-0B58-4213-922A-6EE4F5E15BD3}">
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5734,7 +5094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43106BCE-1E0C-42D9-8C47-8A875A3B9B28}">
   <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -6924,6 +6284,295 @@
       <c r="E71" s="33">
         <v>16</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53C74D93-0A0F-4AF8-A6DA-437C48E3A356}">
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="40.21875" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>388</v>
+      </c>
+      <c r="E1" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="19" t="s">
+        <v>446</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="34">
+        <v>32</v>
+      </c>
+      <c r="D2">
+        <v>70</v>
+      </c>
+      <c r="E2" s="36">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
+        <v>447</v>
+      </c>
+      <c r="B3" s="35"/>
+      <c r="C3" s="34">
+        <v>32</v>
+      </c>
+      <c r="D3">
+        <v>70</v>
+      </c>
+      <c r="E3" s="36">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
+        <v>448</v>
+      </c>
+      <c r="B4" s="35"/>
+      <c r="C4" s="34">
+        <v>30</v>
+      </c>
+      <c r="D4">
+        <v>68</v>
+      </c>
+      <c r="E4" s="36">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
+        <v>449</v>
+      </c>
+      <c r="B5" s="35"/>
+      <c r="C5" s="34">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>68</v>
+      </c>
+      <c r="E5" s="36">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
+        <v>450</v>
+      </c>
+      <c r="B6" s="35"/>
+      <c r="C6" s="34">
+        <v>30</v>
+      </c>
+      <c r="D6">
+        <v>68</v>
+      </c>
+      <c r="E6" s="36">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="s">
+        <v>451</v>
+      </c>
+      <c r="B7" s="35"/>
+      <c r="C7" s="34">
+        <v>30</v>
+      </c>
+      <c r="D7">
+        <v>68</v>
+      </c>
+      <c r="E7" s="36">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
+        <v>452</v>
+      </c>
+      <c r="B8" s="35"/>
+      <c r="C8" s="34">
+        <v>26</v>
+      </c>
+      <c r="D8">
+        <v>62</v>
+      </c>
+      <c r="E8" s="36">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="19" t="s">
+        <v>453</v>
+      </c>
+      <c r="B9" s="35"/>
+      <c r="C9" s="34">
+        <v>26</v>
+      </c>
+      <c r="D9">
+        <v>60</v>
+      </c>
+      <c r="E9" s="36">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="19" t="s">
+        <v>454</v>
+      </c>
+      <c r="B10" s="35"/>
+      <c r="C10" s="34">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>62</v>
+      </c>
+      <c r="E10" s="36">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="19" t="s">
+        <v>455</v>
+      </c>
+      <c r="B11" s="35"/>
+      <c r="C11" s="34">
+        <v>24</v>
+      </c>
+      <c r="D11">
+        <v>60</v>
+      </c>
+      <c r="E11" s="36">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="19" t="s">
+        <v>456</v>
+      </c>
+      <c r="B12" s="35"/>
+      <c r="C12" s="34">
+        <v>25</v>
+      </c>
+      <c r="D12">
+        <v>58</v>
+      </c>
+      <c r="E12" s="36">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="19" t="s">
+        <v>457</v>
+      </c>
+      <c r="B13" s="35"/>
+      <c r="C13" s="34">
+        <v>25</v>
+      </c>
+      <c r="D13">
+        <v>58</v>
+      </c>
+      <c r="E13" s="36">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="19"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="34"/>
+      <c r="E14" s="36"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="19" t="s">
+        <v>458</v>
+      </c>
+      <c r="B15" s="35"/>
+      <c r="C15" s="34"/>
+      <c r="E15" s="36"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="19" t="s">
+        <v>459</v>
+      </c>
+      <c r="B16" s="35"/>
+      <c r="C16" s="34"/>
+      <c r="E16" s="36"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="B17" s="35"/>
+      <c r="C17" s="34"/>
+      <c r="E17" s="36"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="19" t="s">
+        <v>461</v>
+      </c>
+      <c r="B18" s="35"/>
+      <c r="C18" s="34"/>
+      <c r="E18" s="36"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="19"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="34"/>
+      <c r="E19" s="36"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="19" t="s">
+        <v>462</v>
+      </c>
+      <c r="B20" s="35"/>
+      <c r="C20" s="34"/>
+      <c r="E20" s="36"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="19"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="34"/>
+      <c r="E21" s="36"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="19" t="s">
+        <v>463</v>
+      </c>
+      <c r="B22" s="35"/>
+      <c r="C22" s="34"/>
+      <c r="E22" s="36"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="19" t="s">
+        <v>464</v>
+      </c>
+      <c r="B23" s="35"/>
+      <c r="C23" s="34"/>
+      <c r="E23" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12214,15 +11863,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53C74D93-0A0F-4AF8-A6DA-437C48E3A356}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CE67CB9-8D30-45BB-9729-53435DBF7C02}">
   <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -12546,7 +12186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{042C4405-AEC3-4A36-A3E7-7EA75E4B87DD}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -12815,4 +12455,771 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{270FCD42-7C0A-42FB-9872-27F0BB063FAE}">
+  <dimension ref="A1:I32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="6">
+        <v>134</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E2" s="7">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5">
+        <v>99</v>
+      </c>
+      <c r="G2" s="3">
+        <v>107</v>
+      </c>
+      <c r="H2" s="1">
+        <v>37</v>
+      </c>
+      <c r="I2">
+        <f>SUM(D2:H2)*0.55</f>
+        <v>134.255</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="6">
+        <v>144</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="E3" s="7">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>97</v>
+      </c>
+      <c r="G3" s="3">
+        <v>128</v>
+      </c>
+      <c r="H3" s="1">
+        <v>36</v>
+      </c>
+      <c r="I3">
+        <f>SUM(D3:H3)*0.55</f>
+        <v>144.26500000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="6">
+        <v>146</v>
+      </c>
+      <c r="D4" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="E4" s="7">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>97</v>
+      </c>
+      <c r="G4" s="3">
+        <v>132</v>
+      </c>
+      <c r="H4" s="1">
+        <v>36</v>
+      </c>
+      <c r="I4">
+        <f>SUM(D4:H4)*0.55</f>
+        <v>146.46500000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="6">
+        <v>165</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1.4</v>
+      </c>
+      <c r="E5" s="7">
+        <v>0</v>
+      </c>
+      <c r="F5" s="5">
+        <v>96</v>
+      </c>
+      <c r="G5" s="3">
+        <v>142</v>
+      </c>
+      <c r="H5" s="1">
+        <v>35</v>
+      </c>
+      <c r="I5">
+        <f>SUM(D5:H5)*0.6</f>
+        <v>164.64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="6">
+        <v>166</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1.4</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0</v>
+      </c>
+      <c r="F6" s="5">
+        <v>96</v>
+      </c>
+      <c r="G6" s="3">
+        <v>144</v>
+      </c>
+      <c r="H6" s="1">
+        <v>35</v>
+      </c>
+      <c r="I6">
+        <f>SUM(D6:H6)*0.6</f>
+        <v>165.83999999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="6">
+        <v>168</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E7" s="7">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5">
+        <v>95</v>
+      </c>
+      <c r="G7" s="3">
+        <v>149</v>
+      </c>
+      <c r="H7" s="1">
+        <v>34</v>
+      </c>
+      <c r="I7">
+        <f>SUM(D7:H7)*0.6</f>
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="6">
+        <v>229</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5">
+        <v>90</v>
+      </c>
+      <c r="G8" s="3">
+        <v>204</v>
+      </c>
+      <c r="H8" s="1">
+        <v>31</v>
+      </c>
+      <c r="I8">
+        <f>SUM(D8:H8)*0.7</f>
+        <v>228.89999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="6">
+        <v>117</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>100</v>
+      </c>
+      <c r="G9" s="3">
+        <v>95</v>
+      </c>
+      <c r="H9" s="1">
+        <v>38</v>
+      </c>
+      <c r="I9">
+        <f>SUM(D9:H9)*0.5</f>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="6">
+        <v>87</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="7">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>87</v>
+      </c>
+      <c r="G11" s="3">
+        <v>135</v>
+      </c>
+      <c r="H11" s="1">
+        <v>26</v>
+      </c>
+      <c r="I11">
+        <f>SUM(D11:H11)*0.35</f>
+        <v>87.324999999999989</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="6">
+        <v>84</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1.4</v>
+      </c>
+      <c r="E12" s="7">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>88</v>
+      </c>
+      <c r="G12" s="3">
+        <v>126</v>
+      </c>
+      <c r="H12" s="1">
+        <v>25</v>
+      </c>
+      <c r="I12">
+        <f>SUM(D12:H12)*0.35</f>
+        <v>84.14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="6">
+        <v>142</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2</v>
+      </c>
+      <c r="E13" s="7">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5">
+        <v>84</v>
+      </c>
+      <c r="G13" s="3">
+        <v>168</v>
+      </c>
+      <c r="H13" s="1">
+        <v>31</v>
+      </c>
+      <c r="I13">
+        <f>SUM(D13:H13)*0.5</f>
+        <v>142.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="6">
+        <v>285</v>
+      </c>
+      <c r="D15" s="4">
+        <v>3</v>
+      </c>
+      <c r="E15" s="7">
+        <v>9</v>
+      </c>
+      <c r="F15" s="5">
+        <v>84</v>
+      </c>
+      <c r="G15" s="3">
+        <v>355</v>
+      </c>
+      <c r="H15" s="1">
+        <v>25</v>
+      </c>
+      <c r="I15">
+        <f>SUM(D15:H15)*0.6</f>
+        <v>285.59999999999997</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="6">
+        <v>214</v>
+      </c>
+      <c r="D16" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="E16" s="7">
+        <v>9</v>
+      </c>
+      <c r="F16" s="5">
+        <v>92</v>
+      </c>
+      <c r="G16" s="3">
+        <v>175</v>
+      </c>
+      <c r="H16" s="1">
+        <v>27</v>
+      </c>
+      <c r="I16">
+        <f>SUM(D16:H16)*0.7</f>
+        <v>213.85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="6">
+        <v>224</v>
+      </c>
+      <c r="D17" s="4">
+        <v>2.4</v>
+      </c>
+      <c r="E17" s="7">
+        <v>9</v>
+      </c>
+      <c r="F17" s="5">
+        <v>90</v>
+      </c>
+      <c r="G17" s="3">
+        <v>190</v>
+      </c>
+      <c r="H17" s="1">
+        <v>29</v>
+      </c>
+      <c r="I17">
+        <f>SUM(D17:H17)*0.7</f>
+        <v>224.27999999999997</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="6">
+        <v>320</v>
+      </c>
+      <c r="D19" s="4">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E19" s="7">
+        <v>12</v>
+      </c>
+      <c r="F19" s="5">
+        <v>82</v>
+      </c>
+      <c r="G19" s="3">
+        <v>267</v>
+      </c>
+      <c r="H19" s="1">
+        <v>35</v>
+      </c>
+      <c r="I19">
+        <f t="shared" ref="I19:I24" si="0">SUM(D19:H19)*0.8</f>
+        <v>320.32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="6">
+        <v>286</v>
+      </c>
+      <c r="D20" s="4">
+        <v>4</v>
+      </c>
+      <c r="E20" s="7">
+        <v>12</v>
+      </c>
+      <c r="F20" s="5">
+        <v>85</v>
+      </c>
+      <c r="G20" s="3">
+        <v>226</v>
+      </c>
+      <c r="H20" s="1">
+        <v>31</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="0"/>
+        <v>286.40000000000003</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="6">
+        <v>307</v>
+      </c>
+      <c r="D21" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E21" s="7">
+        <v>12</v>
+      </c>
+      <c r="F21" s="5">
+        <v>83</v>
+      </c>
+      <c r="G21" s="3">
+        <v>253</v>
+      </c>
+      <c r="H21" s="1">
+        <v>32</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="0"/>
+        <v>307.36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="6">
+        <v>307</v>
+      </c>
+      <c r="D22" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E22" s="7">
+        <v>12</v>
+      </c>
+      <c r="F22" s="5">
+        <v>83</v>
+      </c>
+      <c r="G22" s="3">
+        <v>253</v>
+      </c>
+      <c r="H22" s="1">
+        <v>32</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="0"/>
+        <v>307.36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="6">
+        <v>308</v>
+      </c>
+      <c r="D23" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E23" s="7">
+        <v>12</v>
+      </c>
+      <c r="F23" s="5">
+        <v>83</v>
+      </c>
+      <c r="G23" s="3">
+        <v>252</v>
+      </c>
+      <c r="H23" s="1">
+        <v>34</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="0"/>
+        <v>308.16000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="6">
+        <v>296</v>
+      </c>
+      <c r="D24" s="4">
+        <v>4.3</v>
+      </c>
+      <c r="E24" s="7">
+        <v>12</v>
+      </c>
+      <c r="F24" s="5">
+        <v>83</v>
+      </c>
+      <c r="G24" s="3">
+        <v>241</v>
+      </c>
+      <c r="H24" s="1">
+        <v>30</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="0"/>
+        <v>296.24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="6">
+        <v>308</v>
+      </c>
+      <c r="D26" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E26" s="7">
+        <v>12</v>
+      </c>
+      <c r="F26" s="5">
+        <v>83</v>
+      </c>
+      <c r="G26" s="3">
+        <v>252</v>
+      </c>
+      <c r="H26" s="1">
+        <v>34</v>
+      </c>
+      <c r="I26">
+        <f>SUM(D26:H26)*0.8</f>
+        <v>308.16000000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="6">
+        <v>308</v>
+      </c>
+      <c r="D27" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E27" s="7">
+        <v>12</v>
+      </c>
+      <c r="F27" s="5">
+        <v>83</v>
+      </c>
+      <c r="G27" s="3">
+        <v>252</v>
+      </c>
+      <c r="H27" s="1">
+        <v>34</v>
+      </c>
+      <c r="I27">
+        <f>SUM(D27:H27)*0.8</f>
+        <v>308.16000000000003</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="6">
+        <v>320</v>
+      </c>
+      <c r="D28" s="4">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E28" s="7">
+        <v>12</v>
+      </c>
+      <c r="F28" s="5">
+        <v>82</v>
+      </c>
+      <c r="G28" s="3">
+        <v>267</v>
+      </c>
+      <c r="H28" s="1">
+        <v>35</v>
+      </c>
+      <c r="I28">
+        <f>SUM(D28:H28)*0.8</f>
+        <v>320.32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B30" s="2"/>
+      <c r="C30" s="6">
+        <v>308</v>
+      </c>
+      <c r="D30" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E30" s="7">
+        <v>12</v>
+      </c>
+      <c r="F30" s="5">
+        <v>83</v>
+      </c>
+      <c r="G30" s="3">
+        <v>252</v>
+      </c>
+      <c r="H30" s="1">
+        <v>34</v>
+      </c>
+      <c r="I30">
+        <f>SUM(D30:H30)*0.8</f>
+        <v>308.16000000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="6">
+        <v>308</v>
+      </c>
+      <c r="D31" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E31" s="7">
+        <v>12</v>
+      </c>
+      <c r="F31" s="5">
+        <v>83</v>
+      </c>
+      <c r="G31" s="3">
+        <v>252</v>
+      </c>
+      <c r="H31" s="1">
+        <v>34</v>
+      </c>
+      <c r="I31">
+        <f>SUM(D31:H31)*0.8</f>
+        <v>308.16000000000003</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="6">
+        <v>308</v>
+      </c>
+      <c r="D32" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E32" s="7">
+        <v>12</v>
+      </c>
+      <c r="F32" s="5">
+        <v>83</v>
+      </c>
+      <c r="G32" s="3">
+        <v>252</v>
+      </c>
+      <c r="H32" s="1">
+        <v>34</v>
+      </c>
+      <c r="I32">
+        <f>SUM(D32:H32)*0.8</f>
+        <v>308.16000000000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>